<commit_message>
Justificación: numerado en el cuerpo en todos los modelos
La captura del proceso de manuales marca que el documento ubica el número del 1 kg en la cúpula y que el
criterio FLAMA es grabarlo en el cuerpo en todos los modelos. Links al commit 8b2bfec.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01E33CYXtZ2f33D1RjoRdR65
</commit_message>
<xml_diff>
--- a/salida/justificacion/Justificacion de medidas planos.xlsx
+++ b/salida/justificacion/Justificacion de medidas planos.xlsx
@@ -24106,7 +24106,7 @@
       </c>
       <c r="D43" s="19" t="inlineStr">
         <is>
-          <t>1: Numerado: desarrollo de 2,5-10 kg; en el 1 kg el número va en la cúpula; 2: Muesca de altura en el cuello (prensa Pannier); 3: Encastre: extremo del cuerpo reducido y fondo encastrado a presión; 4: Bordoneado: bordoneadora SWM-400; profundidad y posición del bordón  — Nota: Documento del usuario (no es la fuente de verdad: se usa para el paso a paso y las medidas que fija).</t>
+          <t>1: Numerado en el cuerpo (desarrollo de 2,5-10 kg). El documento pone el del 1 kg en la cúpula; criterio FLAMA: va en el cuerpo en todos los modelos; 2: Muesca de altura en el cuello (prensa Pannier); 3: Encastre: extremo del cuerpo reducido y fondo encastrado a presión; 4: Bordoneado: bordoneadora SWM-400; profundidad y posición del bordón  — Nota: Documento del usuario (no es la fuente de verdad: se usa para el paso a paso y las medidas que fija).</t>
         </is>
       </c>
       <c r="E43" s="19" t="inlineStr"/>
@@ -24114,7 +24114,7 @@
     <row r="44">
       <c r="A44" s="42" t="inlineStr">
         <is>
-          <t>Valores de diseño FLAMA (amarillo/naranja en las matrices). Links al commit 9cf9127.</t>
+          <t>Valores de diseño FLAMA (amarillo/naranja en las matrices). Links al commit 8b2bfec.</t>
         </is>
       </c>
     </row>
@@ -24342,7 +24342,7 @@
       </c>
       <c r="B53" s="44" t="inlineStr">
         <is>
-          <t>flama/modelo3d.py línea 851</t>
+          <t>flama/modelo3d.py línea 852</t>
         </is>
       </c>
       <c r="C53" s="45" t="inlineStr">

</xml_diff>